<commit_message>
data: weekly EFK refresh (2026-08-15)
</commit_message>
<xml_diff>
--- a/files/exports/de/financings_28_budgetF.xlsx
+++ b/files/exports/de/financings_28_budgetF.xlsx
@@ -354,14 +354,14 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="30.800000000000004" min="1" max="1" bestFit="1" customWidth="1"/>
     <col width="63.800000000000004" min="2" max="2" bestFit="1" customWidth="1"/>
     <col width="14.3" min="3" max="3" bestFit="1" customWidth="1"/>
     <col width="24.75" min="4" max="4" bestFit="1" customWidth="1"/>
-    <col width="56.1" min="5" max="5" bestFit="1" customWidth="1"/>
+    <col width="58.300000000000004" min="5" max="5" bestFit="1" customWidth="1"/>
     <col width="51.7" min="6" max="6" bestFit="1" customWidth="1"/>
     <col width="23.099999999999998" min="7" max="7" bestFit="1" customWidth="1"/>
     <col width="38.5" min="8" max="8" bestFit="1" customWidth="1"/>
@@ -459,7 +459,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3">
-        <v>46241.69967997082</v>
+        <v>46248.61550886367</v>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
@@ -519,7 +519,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3">
-        <v>46241.69967997593</v>
+        <v>46248.615508868745</v>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
@@ -530,11 +530,11 @@
         <v>46187.0</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>374</v>
+        <v>397</v>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Schweizerischer Gewerkschaftsbund (SGB)</t>
+          <t>Travail.Suisse</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="G3" s="6" t="n">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="I3" s="6" t="n">
-        <v>1544</v>
+        <v>1567</v>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
@@ -559,13 +559,13 @@
         </is>
       </c>
       <c r="K3" s="7" t="n">
-        <v>938329.0</v>
+        <v>96175.0</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>844943.0</v>
+        <v>0.0</v>
       </c>
       <c r="M3" s="7" t="n">
-        <v>93386.0</v>
+        <v>0.0</v>
       </c>
       <c r="N3" s="7" t="n">
         <v>0.0</v>
@@ -574,12 +574,12 @@
         <v>0.0</v>
       </c>
       <c r="P3" s="7" t="n">
-        <v>0.0</v>
+        <v>96175.0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3">
-        <v>46241.69967997868</v>
+        <v>46248.6155088714</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
@@ -590,11 +590,11 @@
         <v>46187.0</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>6</v>
+        <v>374</v>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Schweizerische Volkspartei des Kantons Zürich</t>
+          <t>Schweizerischer Gewerkschaftsbund (SGB)</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -603,15 +603,15 @@
         </is>
       </c>
       <c r="G4" s="6" t="n">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Annahme der Abstimmungsvorlage</t>
+          <t>Ablehnung der Abstimmungsvorlage</t>
         </is>
       </c>
       <c r="I4" s="6" t="n">
-        <v>1554</v>
+        <v>1544</v>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
@@ -619,13 +619,13 @@
         </is>
       </c>
       <c r="K4" s="7" t="n">
-        <v>428460.74</v>
+        <v>938329.0</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>108460.74</v>
+        <v>844943.0</v>
       </c>
       <c r="M4" s="7" t="n">
-        <v>0.0</v>
+        <v>93386.0</v>
       </c>
       <c r="N4" s="7" t="n">
         <v>0.0</v>
@@ -634,12 +634,12 @@
         <v>0.0</v>
       </c>
       <c r="P4" s="7" t="n">
-        <v>320000.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3">
-        <v>46241.69967998052</v>
+        <v>46248.61550887321</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
@@ -650,11 +650,11 @@
         <v>46187.0</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>452</v>
+        <v>6</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Allianz für eine funktionierende Schweiz</t>
+          <t>Schweizerische Volkspartei des Kantons Zürich</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -663,15 +663,15 @@
         </is>
       </c>
       <c r="G5" s="6" t="n">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Ablehnung der Abstimmungsvorlage</t>
+          <t>Annahme der Abstimmungsvorlage</t>
         </is>
       </c>
       <c r="I5" s="6" t="n">
-        <v>1541</v>
+        <v>1554</v>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
@@ -679,10 +679,10 @@
         </is>
       </c>
       <c r="K5" s="7" t="n">
-        <v>81900.0</v>
+        <v>428460.74</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>81900.0</v>
+        <v>108460.74</v>
       </c>
       <c r="M5" s="7" t="n">
         <v>0.0</v>
@@ -694,12 +694,12 @@
         <v>0.0</v>
       </c>
       <c r="P5" s="7" t="n">
-        <v>0.0</v>
+        <v>320000.0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3">
-        <v>46241.699679981924</v>
+        <v>46248.61550887459</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
@@ -710,11 +710,11 @@
         <v>46187.0</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>146</v>
+        <v>452</v>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>GastroSuisse</t>
+          <t>Allianz für eine funktionierende Schweiz</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="G6" s="6" t="n">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
@@ -731,7 +731,7 @@
         </is>
       </c>
       <c r="I6" s="6" t="n">
-        <v>1547</v>
+        <v>1541</v>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
@@ -739,13 +739,13 @@
         </is>
       </c>
       <c r="K6" s="7" t="n">
-        <v>133276.59</v>
+        <v>81900.0</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>0.0</v>
+        <v>81900.0</v>
       </c>
       <c r="M6" s="7" t="n">
-        <v>8400.0</v>
+        <v>0.0</v>
       </c>
       <c r="N6" s="7" t="n">
         <v>0.0</v>
@@ -754,12 +754,12 @@
         <v>0.0</v>
       </c>
       <c r="P6" s="7" t="n">
-        <v>124876.59</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3">
-        <v>46241.699679983256</v>
+        <v>46248.61550887584</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
@@ -770,50 +770,710 @@
         <v>46187.0</v>
       </c>
       <c r="D7" s="6" t="n">
+        <v>380</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Gewerkschaft Unia</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>572</v>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>1578</v>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung der Schlussrechnung über die Einnahmen</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="n">
+        <v>239386.94</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <v>19985.35</v>
+      </c>
+      <c r="M7" s="7" t="n">
+        <v>108500.0</v>
+      </c>
+      <c r="N7" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="O7" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="P7" s="7" t="n">
+        <v>110901.59</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>46248.6155088773</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C8" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>453</v>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Tourismuskomitee</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>573</v>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>1562</v>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung der Schlussrechnung über die Einnahmen</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>130000.0</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <v>130000.0</v>
+      </c>
+      <c r="M8" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N8" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="O8" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="P8" s="7" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3">
+        <v>46248.615508879404</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C9" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>146</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>GastroSuisse</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>574</v>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>1547</v>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung der Schlussrechnung über die Einnahmen</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>133276.59</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>8400.0</v>
+      </c>
+      <c r="N9" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="O9" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="P9" s="7" t="n">
+        <v>124876.59</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3">
+        <v>46248.61550888153</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C10" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>406</v>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>SMV Schweizerischer Mieterinnen- und Mieterverband</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>576</v>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>1568</v>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung der Schlussrechnung über die Einnahmen</t>
+        </is>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>98412.0</v>
+      </c>
+      <c r="L10" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M10" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N10" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="O10" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="P10" s="7" t="n">
+        <v>98412.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3">
+        <v>46248.61550888302</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C11" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>FDP.Die Liberalen</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>577</v>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>1569</v>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung der Schlussrechnung über die Einnahmen</t>
+        </is>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>195520.0</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <v>195520.0</v>
+      </c>
+      <c r="M11" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N11" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="O11" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="P11" s="7" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3">
+        <v>46248.615508884344</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C12" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>454</v>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Allianz "Nein zur Chaos-Initiative"</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>578</v>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>1576</v>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung der Schlussrechnung über die Einnahmen</t>
+        </is>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>4768845.0</v>
+      </c>
+      <c r="L12" s="7" t="n">
+        <v>4563858.0</v>
+      </c>
+      <c r="M12" s="7" t="n">
+        <v>204987.0</v>
+      </c>
+      <c r="N12" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="O12" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="P12" s="7" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3">
+        <v>46248.615508885574</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C13" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>418</v>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>IG Nachhaltigkeitsinitiative</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>579</v>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Annahme der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>1555</v>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung der Schlussrechnung über die Einnahmen</t>
+        </is>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>6173061.58</v>
+      </c>
+      <c r="L13" s="7" t="n">
+        <v>5678238.72</v>
+      </c>
+      <c r="M13" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N13" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="O13" s="7" t="n">
+        <v>93822.0</v>
+      </c>
+      <c r="P13" s="7" t="n">
+        <v>401000.86</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3">
+        <v>46248.61550888676</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C14" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Sozialdemokratische Partei der Schweiz</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>580</v>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>1563</v>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung der Schlussrechnung über die Einnahmen</t>
+        </is>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>1901724.0</v>
+      </c>
+      <c r="L14" s="7" t="n">
+        <v>1890880.0</v>
+      </c>
+      <c r="M14" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N14" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="O14" s="7" t="n">
+        <v>10844.0</v>
+      </c>
+      <c r="P14" s="7" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3">
+        <v>46248.61550888791</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C15" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Die Mitte</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>582</v>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>1566</v>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung der Schlussrechnung über die Einnahmen</t>
+        </is>
+      </c>
+      <c r="K15" s="7" t="n">
+        <v>135000.0</v>
+      </c>
+      <c r="L15" s="7" t="n">
+        <v>135000.0</v>
+      </c>
+      <c r="M15" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N15" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="O15" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="P15" s="7" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3">
+        <v>46248.61550888943</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C16" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>413</v>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Handel Schweiz</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>586</v>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>1583</v>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung der Schlussrechnung über die Einnahmen</t>
+        </is>
+      </c>
+      <c r="K16" s="7" t="n">
+        <v>91724.0</v>
+      </c>
+      <c r="L16" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M16" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N16" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="O16" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="P16" s="7" t="n">
+        <v>91724.0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3">
+        <v>46248.615508891016</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C17" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>458</v>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Schweizer Hotelier-Verein (SHV)</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>587</v>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>1584</v>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung der Schlussrechnung über die Einnahmen</t>
+        </is>
+      </c>
+      <c r="K17" s="7" t="n">
+        <v>89311.85</v>
+      </c>
+      <c r="L17" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M17" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N17" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="O17" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="P17" s="7" t="n">
+        <v>89311.85</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3">
+        <v>46248.61550889264</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C18" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D18" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>Sozialdemokratische Partei des Kantons Zürich</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Juristische Person oder Personengesellschaft</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="n">
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="n">
         <v>588</v>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>Ablehnung der Abstimmungsvorlage</t>
         </is>
       </c>
-      <c r="I7" s="6" t="n">
+      <c r="I18" s="6" t="n">
         <v>1549</v>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="J18" s="4" t="inlineStr">
         <is>
           <t>Offenlegung der Schlussrechnung über die Einnahmen</t>
         </is>
       </c>
-      <c r="K7" s="7" t="n">
+      <c r="K18" s="7" t="n">
         <v>68602.3</v>
       </c>
-      <c r="L7" s="7" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="M7" s="7" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N7" s="7" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="O7" s="7" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="P7" s="7" t="n">
+      <c r="L18" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M18" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N18" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="O18" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="P18" s="7" t="n">
         <v>68602.3</v>
       </c>
     </row>
@@ -831,7 +1491,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:V34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="30.800000000000004" min="1" max="1" bestFit="1" customWidth="1"/>
@@ -849,11 +1509,11 @@
     <col width="61.05" min="13" max="13" bestFit="1" customWidth="1"/>
     <col width="31.349999999999998" min="14" max="14" bestFit="1" customWidth="1"/>
     <col width="36.3" min="15" max="15" bestFit="1" customWidth="1"/>
-    <col width="57.75" min="16" max="16" bestFit="1" customWidth="1"/>
+    <col width="67.10000000000001" min="16" max="16" bestFit="1" customWidth="1"/>
     <col width="51.15" min="17" max="17" bestFit="1" customWidth="1"/>
     <col width="33.0" min="18" max="18" bestFit="1" customWidth="1"/>
     <col width="31.349999999999998" min="19" max="19" bestFit="1" customWidth="1"/>
-    <col width="48.400000000000006" min="20" max="20" bestFit="1" customWidth="1"/>
+    <col width="68.2" min="20" max="20" bestFit="1" customWidth="1"/>
     <col width="26.4" min="21" max="21" bestFit="1" customWidth="1"/>
     <col width="52.8" min="22" max="22" bestFit="1" customWidth="1"/>
   </cols>
@@ -972,7 +1632,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3">
-        <v>46241.69967998607</v>
+        <v>46248.615508895775</v>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
@@ -1044,7 +1704,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3">
-        <v>46241.69967998787</v>
+        <v>46248.615508897645</v>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
@@ -1116,7 +1776,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3">
-        <v>46241.69967998934</v>
+        <v>46248.615508898845</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
@@ -1188,7 +1848,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3">
-        <v>46241.69967999031</v>
+        <v>46248.61550889978</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
@@ -1260,7 +1920,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3">
-        <v>46241.69967999123</v>
+        <v>46248.61550890088</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
@@ -1340,7 +2000,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3">
-        <v>46241.69967999228</v>
+        <v>46248.615508902054</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
@@ -1408,6 +2068,1998 @@
       </c>
       <c r="V7" s="5">
         <v>46212.0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>46248.61550890322</v>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C8" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>380</v>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Gewerkschaft Unia</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>572</v>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>1579</v>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>4578</v>
+      </c>
+      <c r="L8" s="4"/>
+      <c r="M8" s="4"/>
+      <c r="N8" s="4"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4" t="inlineStr">
+        <is>
+          <t>Gewerkschaft Unia</t>
+        </is>
+      </c>
+      <c r="Q8" s="4" t="inlineStr">
+        <is>
+          <t>Bern</t>
+        </is>
+      </c>
+      <c r="R8" s="4" t="inlineStr">
+        <is>
+          <t>Nichtmonetär</t>
+        </is>
+      </c>
+      <c r="S8" s="4" t="inlineStr">
+        <is>
+          <t>Dienstleistung</t>
+        </is>
+      </c>
+      <c r="T8" s="4" t="inlineStr">
+        <is>
+          <t>Arbeitsaufwand von Unia-Mitarbeitenden (bezahlt über Löhne)</t>
+        </is>
+      </c>
+      <c r="U8" s="7" t="n">
+        <v>108500.0</v>
+      </c>
+      <c r="V8" s="5">
+        <v>46187.0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3">
+        <v>46248.61550890416</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C9" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>453</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Tourismuskomitee</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>573</v>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>1543</v>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>4501</v>
+      </c>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4" t="inlineStr">
+        <is>
+          <t>Schweizer Tourismus-Verband</t>
+        </is>
+      </c>
+      <c r="Q9" s="4" t="inlineStr">
+        <is>
+          <t>Bern</t>
+        </is>
+      </c>
+      <c r="R9" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S9" s="4"/>
+      <c r="T9" s="4"/>
+      <c r="U9" s="7" t="n">
+        <v>50000.0</v>
+      </c>
+      <c r="V9" s="5">
+        <v>46097.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3">
+        <v>46248.61550890552</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C10" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>453</v>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Tourismuskomitee</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>573</v>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>1543</v>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>4502</v>
+      </c>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="4" t="inlineStr">
+        <is>
+          <t>economiesuisse</t>
+        </is>
+      </c>
+      <c r="Q10" s="4" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+      <c r="R10" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S10" s="4"/>
+      <c r="T10" s="4"/>
+      <c r="U10" s="7" t="n">
+        <v>50000.0</v>
+      </c>
+      <c r="V10" s="5">
+        <v>46188.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3">
+        <v>46248.61550890638</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C11" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>453</v>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Tourismuskomitee</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>573</v>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>1543</v>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>4503</v>
+      </c>
+      <c r="L11" s="4"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="4"/>
+      <c r="P11" s="4" t="inlineStr">
+        <is>
+          <t>HotellerieSuisse</t>
+        </is>
+      </c>
+      <c r="Q11" s="4" t="inlineStr">
+        <is>
+          <t>Bern</t>
+        </is>
+      </c>
+      <c r="R11" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S11" s="4"/>
+      <c r="T11" s="4"/>
+      <c r="U11" s="7" t="n">
+        <v>15000.0</v>
+      </c>
+      <c r="V11" s="5">
+        <v>46139.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3">
+        <v>46248.61550890722</v>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C12" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>453</v>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Tourismuskomitee</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>573</v>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>1543</v>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>4504</v>
+      </c>
+      <c r="L12" s="4"/>
+      <c r="M12" s="4"/>
+      <c r="N12" s="4"/>
+      <c r="O12" s="4"/>
+      <c r="P12" s="4" t="inlineStr">
+        <is>
+          <t>GastroSuisse</t>
+        </is>
+      </c>
+      <c r="Q12" s="4" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+      <c r="R12" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S12" s="4"/>
+      <c r="T12" s="4"/>
+      <c r="U12" s="7" t="n">
+        <v>15000.0</v>
+      </c>
+      <c r="V12" s="5">
+        <v>46142.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3">
+        <v>46248.61550890806</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C13" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>FDP.Die Liberalen</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>577</v>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>1570</v>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K13" s="6" t="n">
+        <v>4563</v>
+      </c>
+      <c r="L13" s="4"/>
+      <c r="M13" s="4"/>
+      <c r="N13" s="4"/>
+      <c r="O13" s="4"/>
+      <c r="P13" s="4" t="inlineStr">
+        <is>
+          <t>economiesuisse</t>
+        </is>
+      </c>
+      <c r="Q13" s="4" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+      <c r="R13" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S13" s="4"/>
+      <c r="T13" s="4"/>
+      <c r="U13" s="7" t="n">
+        <v>130000.0</v>
+      </c>
+      <c r="V13" s="5">
+        <v>46188.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3">
+        <v>46248.61550890893</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C14" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>FDP.Die Liberalen</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>577</v>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>1570</v>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K14" s="6" t="n">
+        <v>4564</v>
+      </c>
+      <c r="L14" s="4"/>
+      <c r="M14" s="4"/>
+      <c r="N14" s="4"/>
+      <c r="O14" s="4"/>
+      <c r="P14" s="4" t="inlineStr">
+        <is>
+          <t>economiesuisse</t>
+        </is>
+      </c>
+      <c r="Q14" s="4" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+      <c r="R14" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S14" s="4"/>
+      <c r="T14" s="4"/>
+      <c r="U14" s="7" t="n">
+        <v>50000.0</v>
+      </c>
+      <c r="V14" s="5">
+        <v>46188.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3">
+        <v>46248.615508909854</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C15" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>FDP.Die Liberalen</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>577</v>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>1570</v>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>4565</v>
+      </c>
+      <c r="L15" s="4"/>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4"/>
+      <c r="O15" s="4"/>
+      <c r="P15" s="4" t="inlineStr">
+        <is>
+          <t>economiesuisse</t>
+        </is>
+      </c>
+      <c r="Q15" s="4" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+      <c r="R15" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S15" s="4"/>
+      <c r="T15" s="4"/>
+      <c r="U15" s="7" t="n">
+        <v>5000.0</v>
+      </c>
+      <c r="V15" s="5">
+        <v>46197.0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3">
+        <v>46248.61550891075</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C16" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>454</v>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Allianz "Nein zur Chaos-Initiative"</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>578</v>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>1577</v>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K16" s="6" t="n">
+        <v>4600</v>
+      </c>
+      <c r="L16" s="4"/>
+      <c r="M16" s="4"/>
+      <c r="N16" s="4"/>
+      <c r="O16" s="4"/>
+      <c r="P16" s="4" t="inlineStr">
+        <is>
+          <t>Handelskammer beider Basel</t>
+        </is>
+      </c>
+      <c r="Q16" s="4" t="inlineStr">
+        <is>
+          <t>Basel</t>
+        </is>
+      </c>
+      <c r="R16" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S16" s="4"/>
+      <c r="T16" s="4"/>
+      <c r="U16" s="7" t="n">
+        <v>20000.0</v>
+      </c>
+      <c r="V16" s="5">
+        <v>46120.0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3">
+        <v>46248.61550891163</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C17" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>454</v>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Allianz "Nein zur Chaos-Initiative"</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>578</v>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>1577</v>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K17" s="6" t="n">
+        <v>4601</v>
+      </c>
+      <c r="L17" s="4"/>
+      <c r="M17" s="4"/>
+      <c r="N17" s="4"/>
+      <c r="O17" s="4"/>
+      <c r="P17" s="4" t="inlineStr">
+        <is>
+          <t>Fédération des Entreprises Romandes Genève</t>
+        </is>
+      </c>
+      <c r="Q17" s="4" t="inlineStr">
+        <is>
+          <t>Genève</t>
+        </is>
+      </c>
+      <c r="R17" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S17" s="4"/>
+      <c r="T17" s="4"/>
+      <c r="U17" s="7" t="n">
+        <v>78719.0</v>
+      </c>
+      <c r="V17" s="5">
+        <v>46136.0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3">
+        <v>46248.61550891261</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C18" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>454</v>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Allianz "Nein zur Chaos-Initiative"</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>578</v>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>1577</v>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K18" s="6" t="n">
+        <v>4602</v>
+      </c>
+      <c r="L18" s="4"/>
+      <c r="M18" s="4"/>
+      <c r="N18" s="4"/>
+      <c r="O18" s="4"/>
+      <c r="P18" s="4" t="inlineStr">
+        <is>
+          <t>Groupement des Entreprises Multinationales</t>
+        </is>
+      </c>
+      <c r="Q18" s="4" t="inlineStr">
+        <is>
+          <t>Genève</t>
+        </is>
+      </c>
+      <c r="R18" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S18" s="4"/>
+      <c r="T18" s="4"/>
+      <c r="U18" s="7" t="n">
+        <v>46000.0</v>
+      </c>
+      <c r="V18" s="5">
+        <v>46136.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3">
+        <v>46248.6155089135</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C19" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>454</v>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Allianz "Nein zur Chaos-Initiative"</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>578</v>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="n">
+        <v>1577</v>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K19" s="6" t="n">
+        <v>4603</v>
+      </c>
+      <c r="L19" s="4"/>
+      <c r="M19" s="4"/>
+      <c r="N19" s="4"/>
+      <c r="O19" s="4"/>
+      <c r="P19" s="4" t="inlineStr">
+        <is>
+          <t>Chambre de commerce, d’industrie et des services de Genève</t>
+        </is>
+      </c>
+      <c r="Q19" s="4" t="inlineStr">
+        <is>
+          <t>Genève</t>
+        </is>
+      </c>
+      <c r="R19" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S19" s="4"/>
+      <c r="T19" s="4"/>
+      <c r="U19" s="7" t="n">
+        <v>40000.0</v>
+      </c>
+      <c r="V19" s="5">
+        <v>46136.0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3">
+        <v>46248.61550891433</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C20" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>454</v>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Allianz "Nein zur Chaos-Initiative"</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>578</v>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>1577</v>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K20" s="6" t="n">
+        <v>4604</v>
+      </c>
+      <c r="L20" s="4"/>
+      <c r="M20" s="4"/>
+      <c r="N20" s="4"/>
+      <c r="O20" s="4"/>
+      <c r="P20" s="4" t="inlineStr">
+        <is>
+          <t>Zürcher Handelskammer</t>
+        </is>
+      </c>
+      <c r="Q20" s="4" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+      <c r="R20" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S20" s="4"/>
+      <c r="T20" s="4"/>
+      <c r="U20" s="7" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="V20" s="5">
+        <v>46126.0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3">
+        <v>46248.61550891521</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C21" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>454</v>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Allianz "Nein zur Chaos-Initiative"</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>578</v>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="n">
+        <v>1577</v>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K21" s="6" t="n">
+        <v>4605</v>
+      </c>
+      <c r="L21" s="4"/>
+      <c r="M21" s="4"/>
+      <c r="N21" s="4"/>
+      <c r="O21" s="4"/>
+      <c r="P21" s="4" t="inlineStr">
+        <is>
+          <t>economiesuisse</t>
+        </is>
+      </c>
+      <c r="Q21" s="4" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+      <c r="R21" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S21" s="4"/>
+      <c r="T21" s="4"/>
+      <c r="U21" s="7" t="n">
+        <v>3720000.0</v>
+      </c>
+      <c r="V21" s="5">
+        <v>45987.0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3">
+        <v>46248.6155089162</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C22" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>454</v>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Allianz "Nein zur Chaos-Initiative"</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>578</v>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="n">
+        <v>1577</v>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K22" s="6" t="n">
+        <v>4606</v>
+      </c>
+      <c r="L22" s="4"/>
+      <c r="M22" s="4"/>
+      <c r="N22" s="4"/>
+      <c r="O22" s="4"/>
+      <c r="P22" s="4" t="inlineStr">
+        <is>
+          <t>economiesuisse</t>
+        </is>
+      </c>
+      <c r="Q22" s="4" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+      <c r="R22" s="4" t="inlineStr">
+        <is>
+          <t>Nichtmonetär</t>
+        </is>
+      </c>
+      <c r="S22" s="4" t="inlineStr">
+        <is>
+          <t>Dienstleistung</t>
+        </is>
+      </c>
+      <c r="T22" s="4" t="inlineStr">
+        <is>
+          <t>Löhne</t>
+        </is>
+      </c>
+      <c r="U22" s="7" t="n">
+        <v>196560.0</v>
+      </c>
+      <c r="V22" s="5">
+        <v>46142.0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3">
+        <v>46248.61550891715</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C23" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>454</v>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Allianz "Nein zur Chaos-Initiative"</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>578</v>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="n">
+        <v>1577</v>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K23" s="6" t="n">
+        <v>4607</v>
+      </c>
+      <c r="L23" s="4"/>
+      <c r="M23" s="4"/>
+      <c r="N23" s="4"/>
+      <c r="O23" s="4"/>
+      <c r="P23" s="4" t="inlineStr">
+        <is>
+          <t>economiesuisse</t>
+        </is>
+      </c>
+      <c r="Q23" s="4" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+      <c r="R23" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S23" s="4"/>
+      <c r="T23" s="4"/>
+      <c r="U23" s="7" t="n">
+        <v>420000.0</v>
+      </c>
+      <c r="V23" s="5">
+        <v>46147.0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3">
+        <v>46248.61550891801</v>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C24" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>454</v>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Allianz "Nein zur Chaos-Initiative"</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>578</v>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="n">
+        <v>1577</v>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K24" s="6" t="n">
+        <v>4608</v>
+      </c>
+      <c r="L24" s="4"/>
+      <c r="M24" s="4"/>
+      <c r="N24" s="4"/>
+      <c r="O24" s="4"/>
+      <c r="P24" s="4" t="inlineStr">
+        <is>
+          <t>Fondation Genève Place Financière</t>
+        </is>
+      </c>
+      <c r="Q24" s="4" t="inlineStr">
+        <is>
+          <t>Genève</t>
+        </is>
+      </c>
+      <c r="R24" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S24" s="4"/>
+      <c r="T24" s="4"/>
+      <c r="U24" s="7" t="n">
+        <v>45000.0</v>
+      </c>
+      <c r="V24" s="5">
+        <v>46143.0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3">
+        <v>46248.615508918854</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C25" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>418</v>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>IG Nachhaltigkeitsinitiative</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>579</v>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Annahme der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="n">
+        <v>1556</v>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K25" s="6" t="n">
+        <v>4531</v>
+      </c>
+      <c r="L25" s="4"/>
+      <c r="M25" s="4"/>
+      <c r="N25" s="4"/>
+      <c r="O25" s="4"/>
+      <c r="P25" s="4" t="inlineStr">
+        <is>
+          <t>Schweizerische Volkspartei des Kantons Zürich</t>
+        </is>
+      </c>
+      <c r="Q25" s="4" t="inlineStr">
+        <is>
+          <t>Dübendorf</t>
+        </is>
+      </c>
+      <c r="R25" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S25" s="4"/>
+      <c r="T25" s="4"/>
+      <c r="U25" s="7" t="n">
+        <v>814753.51</v>
+      </c>
+      <c r="V25" s="5">
+        <v>46223.0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3">
+        <v>46248.61550891975</v>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C26" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>418</v>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>IG Nachhaltigkeitsinitiative</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>579</v>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>Annahme der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="n">
+        <v>1556</v>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K26" s="6" t="n">
+        <v>4532</v>
+      </c>
+      <c r="L26" s="4"/>
+      <c r="M26" s="4"/>
+      <c r="N26" s="4"/>
+      <c r="O26" s="4"/>
+      <c r="P26" s="4" t="inlineStr">
+        <is>
+          <t>Stiftung für bürgerliche Politik</t>
+        </is>
+      </c>
+      <c r="Q26" s="4" t="inlineStr">
+        <is>
+          <t>Zug</t>
+        </is>
+      </c>
+      <c r="R26" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S26" s="4"/>
+      <c r="T26" s="4"/>
+      <c r="U26" s="7" t="n">
+        <v>1050000.0</v>
+      </c>
+      <c r="V26" s="5">
+        <v>46176.0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3">
+        <v>46248.61550892061</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C27" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>418</v>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>IG Nachhaltigkeitsinitiative</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>579</v>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>Annahme der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="n">
+        <v>1556</v>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K27" s="6" t="n">
+        <v>4533</v>
+      </c>
+      <c r="L27" s="4"/>
+      <c r="M27" s="4"/>
+      <c r="N27" s="4"/>
+      <c r="O27" s="4"/>
+      <c r="P27" s="4" t="inlineStr">
+        <is>
+          <t>Schweizerische Volkspartei (SVP Schweiz)</t>
+        </is>
+      </c>
+      <c r="Q27" s="4" t="inlineStr">
+        <is>
+          <t>Bern</t>
+        </is>
+      </c>
+      <c r="R27" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S27" s="4"/>
+      <c r="T27" s="4"/>
+      <c r="U27" s="7" t="n">
+        <v>2700000.0</v>
+      </c>
+      <c r="V27" s="5">
+        <v>46195.0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3">
+        <v>46248.6155089216</v>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C28" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>418</v>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>IG Nachhaltigkeitsinitiative</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>579</v>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>Annahme der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="n">
+        <v>1556</v>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K28" s="6" t="n">
+        <v>4534</v>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Blocher</t>
+        </is>
+      </c>
+      <c r="M28" s="4" t="inlineStr">
+        <is>
+          <t>Christoph</t>
+        </is>
+      </c>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t>Herrliberg</t>
+        </is>
+      </c>
+      <c r="O28" s="4" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="P28" s="4"/>
+      <c r="Q28" s="4"/>
+      <c r="R28" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S28" s="4"/>
+      <c r="T28" s="4"/>
+      <c r="U28" s="7" t="n">
+        <v>133332.65</v>
+      </c>
+      <c r="V28" s="5">
+        <v>46197.0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3">
+        <v>46248.61550892257</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C29" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>418</v>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>IG Nachhaltigkeitsinitiative</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>579</v>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>Annahme der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="n">
+        <v>1556</v>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K29" s="6" t="n">
+        <v>4535</v>
+      </c>
+      <c r="L29" s="4"/>
+      <c r="M29" s="4"/>
+      <c r="N29" s="4"/>
+      <c r="O29" s="4"/>
+      <c r="P29" s="4" t="inlineStr">
+        <is>
+          <t>Emil Frey AG</t>
+        </is>
+      </c>
+      <c r="Q29" s="4" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+      <c r="R29" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S29" s="4"/>
+      <c r="T29" s="4"/>
+      <c r="U29" s="7" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="V29" s="5">
+        <v>46077.0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3">
+        <v>46248.615508923525</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C30" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>418</v>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>IG Nachhaltigkeitsinitiative</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>579</v>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>Annahme der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="n">
+        <v>1556</v>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K30" s="6" t="n">
+        <v>4539</v>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>Gaydoul</t>
+        </is>
+      </c>
+      <c r="M30" s="4" t="inlineStr">
+        <is>
+          <t>Philippe</t>
+        </is>
+      </c>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>Küsnacht</t>
+        </is>
+      </c>
+      <c r="O30" s="4" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="P30" s="4"/>
+      <c r="Q30" s="4"/>
+      <c r="R30" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S30" s="4"/>
+      <c r="T30" s="4"/>
+      <c r="U30" s="7" t="n">
+        <v>250000.0</v>
+      </c>
+      <c r="V30" s="5">
+        <v>45832.0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3">
+        <v>46248.61550892445</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C31" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>418</v>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>IG Nachhaltigkeitsinitiative</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>579</v>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>Annahme der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="n">
+        <v>1556</v>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K31" s="6" t="n">
+        <v>4541</v>
+      </c>
+      <c r="L31" s="4"/>
+      <c r="M31" s="4"/>
+      <c r="N31" s="4"/>
+      <c r="O31" s="4"/>
+      <c r="P31" s="4" t="inlineStr">
+        <is>
+          <t>Patinex AG</t>
+        </is>
+      </c>
+      <c r="Q31" s="4" t="inlineStr">
+        <is>
+          <t>Freienbach</t>
+        </is>
+      </c>
+      <c r="R31" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S31" s="4"/>
+      <c r="T31" s="4"/>
+      <c r="U31" s="7" t="n">
+        <v>100000.0</v>
+      </c>
+      <c r="V31" s="5">
+        <v>46160.0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3">
+        <v>46248.61550892531</v>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C32" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Sozialdemokratische Partei der Schweiz</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>580</v>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="n">
+        <v>1564</v>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K32" s="6" t="n">
+        <v>4550</v>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>Brändlin</t>
+        </is>
+      </c>
+      <c r="M32" s="4" t="inlineStr">
+        <is>
+          <t>Sabine und Dominik</t>
+        </is>
+      </c>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t>Liestal</t>
+        </is>
+      </c>
+      <c r="O32" s="4" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="P32" s="4"/>
+      <c r="Q32" s="4"/>
+      <c r="R32" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S32" s="4"/>
+      <c r="T32" s="4"/>
+      <c r="U32" s="7" t="n">
+        <v>20000.0</v>
+      </c>
+      <c r="V32" s="5">
+        <v>46154.0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3">
+        <v>46248.61550892622</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C33" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Sozialdemokratische Partei der Schweiz</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="n">
+        <v>580</v>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="n">
+        <v>1564</v>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K33" s="6" t="n">
+        <v>4551</v>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Murbach und Nussbaum</t>
+        </is>
+      </c>
+      <c r="M33" s="4" t="inlineStr">
+        <is>
+          <t>Urs und Theresa</t>
+        </is>
+      </c>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t>Au</t>
+        </is>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="P33" s="4"/>
+      <c r="Q33" s="4"/>
+      <c r="R33" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S33" s="4"/>
+      <c r="T33" s="4"/>
+      <c r="U33" s="7" t="n">
+        <v>40000.0</v>
+      </c>
+      <c r="V33" s="5">
+        <v>46148.0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3">
+        <v>46248.61550892714</v>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C34" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D34" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Die Mitte</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v>582</v>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="n">
+        <v>1565</v>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung von Zuwendungen über 15 000 Franken (Schlussrechnung)</t>
+        </is>
+      </c>
+      <c r="K34" s="6" t="n">
+        <v>4589</v>
+      </c>
+      <c r="L34" s="4"/>
+      <c r="M34" s="4"/>
+      <c r="N34" s="4"/>
+      <c r="O34" s="4"/>
+      <c r="P34" s="4" t="inlineStr">
+        <is>
+          <t>Economiesuisse</t>
+        </is>
+      </c>
+      <c r="Q34" s="4" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+      <c r="R34" s="4" t="inlineStr">
+        <is>
+          <t>Monetär</t>
+        </is>
+      </c>
+      <c r="S34" s="4"/>
+      <c r="T34" s="4"/>
+      <c r="U34" s="7" t="n">
+        <v>135000.0</v>
+      </c>
+      <c r="V34" s="5">
+        <v>46247.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: weekly EFK refresh (2026-08-22)
</commit_message>
<xml_diff>
--- a/files/exports/de/financings_28_budgetF.xlsx
+++ b/files/exports/de/financings_28_budgetF.xlsx
@@ -354,7 +354,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="30.800000000000004" min="1" max="1" bestFit="1" customWidth="1"/>
@@ -459,7 +459,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3">
-        <v>46248.61550886367</v>
+        <v>46255.35675358324</v>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
@@ -519,7 +519,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3">
-        <v>46248.615508868745</v>
+        <v>46255.35675358769</v>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
@@ -579,7 +579,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3">
-        <v>46248.6155088714</v>
+        <v>46255.35675358963</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
@@ -639,7 +639,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3">
-        <v>46248.61550887321</v>
+        <v>46255.356753591244</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
@@ -699,7 +699,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3">
-        <v>46248.61550887459</v>
+        <v>46255.35675359327</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
@@ -759,7 +759,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3">
-        <v>46248.61550887584</v>
+        <v>46255.35675359503</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
@@ -819,7 +819,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3">
-        <v>46248.6155088773</v>
+        <v>46255.35675359662</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
@@ -879,7 +879,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3">
-        <v>46248.615508879404</v>
+        <v>46255.356753598615</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3">
-        <v>46248.61550888153</v>
+        <v>46255.35675360019</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
@@ -950,11 +950,11 @@
         <v>46187.0</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>406</v>
+        <v>357</v>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>SMV Schweizerischer Mieterinnen- und Mieterverband</t>
+          <t>Operation Libero</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="G10" s="6" t="n">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="I10" s="6" t="n">
-        <v>1568</v>
+        <v>1582</v>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
@@ -979,27 +979,27 @@
         </is>
       </c>
       <c r="K10" s="7" t="n">
-        <v>98412.0</v>
+        <v>279737.09</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>0.0</v>
+        <v>258122.7</v>
       </c>
       <c r="M10" s="7" t="n">
         <v>0.0</v>
       </c>
       <c r="N10" s="7" t="n">
-        <v>0.0</v>
+        <v>551.39</v>
       </c>
       <c r="O10" s="7" t="n">
-        <v>0.0</v>
+        <v>21063.0</v>
       </c>
       <c r="P10" s="7" t="n">
-        <v>98412.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3">
-        <v>46248.61550888302</v>
+        <v>46255.35675360173</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
@@ -1010,11 +1010,11 @@
         <v>46187.0</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>43</v>
+        <v>406</v>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>FDP.Die Liberalen</t>
+          <t>SMV Schweizerischer Mieterinnen- und Mieterverband</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -1023,7 +1023,7 @@
         </is>
       </c>
       <c r="G11" s="6" t="n">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
@@ -1031,7 +1031,7 @@
         </is>
       </c>
       <c r="I11" s="6" t="n">
-        <v>1569</v>
+        <v>1568</v>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
@@ -1039,10 +1039,10 @@
         </is>
       </c>
       <c r="K11" s="7" t="n">
-        <v>195520.0</v>
+        <v>98412.0</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>195520.0</v>
+        <v>0.0</v>
       </c>
       <c r="M11" s="7" t="n">
         <v>0.0</v>
@@ -1054,12 +1054,12 @@
         <v>0.0</v>
       </c>
       <c r="P11" s="7" t="n">
-        <v>0.0</v>
+        <v>98412.0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3">
-        <v>46248.615508884344</v>
+        <v>46255.356753603264</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
@@ -1070,11 +1070,11 @@
         <v>46187.0</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>454</v>
+        <v>43</v>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Allianz "Nein zur Chaos-Initiative"</t>
+          <t>FDP.Die Liberalen</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -1083,7 +1083,7 @@
         </is>
       </c>
       <c r="G12" s="6" t="n">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="I12" s="6" t="n">
-        <v>1576</v>
+        <v>1569</v>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
@@ -1099,13 +1099,13 @@
         </is>
       </c>
       <c r="K12" s="7" t="n">
-        <v>4768845.0</v>
+        <v>195520.0</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>4563858.0</v>
+        <v>195520.0</v>
       </c>
       <c r="M12" s="7" t="n">
-        <v>204987.0</v>
+        <v>0.0</v>
       </c>
       <c r="N12" s="7" t="n">
         <v>0.0</v>
@@ -1119,7 +1119,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3">
-        <v>46248.615508885574</v>
+        <v>46255.35675360513</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
@@ -1130,11 +1130,11 @@
         <v>46187.0</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>418</v>
+        <v>454</v>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>IG Nachhaltigkeitsinitiative</t>
+          <t>Allianz "Nein zur Chaos-Initiative"</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -1143,15 +1143,15 @@
         </is>
       </c>
       <c r="G13" s="6" t="n">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Annahme der Abstimmungsvorlage</t>
+          <t>Ablehnung der Abstimmungsvorlage</t>
         </is>
       </c>
       <c r="I13" s="6" t="n">
-        <v>1555</v>
+        <v>1576</v>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
@@ -1159,27 +1159,27 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>6173061.58</v>
+        <v>4768845.0</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>5678238.72</v>
+        <v>4563858.0</v>
       </c>
       <c r="M13" s="7" t="n">
-        <v>0.0</v>
+        <v>204987.0</v>
       </c>
       <c r="N13" s="7" t="n">
         <v>0.0</v>
       </c>
       <c r="O13" s="7" t="n">
-        <v>93822.0</v>
+        <v>0.0</v>
       </c>
       <c r="P13" s="7" t="n">
-        <v>401000.86</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3">
-        <v>46248.61550888676</v>
+        <v>46255.356753606684</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
@@ -1190,11 +1190,11 @@
         <v>46187.0</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>8</v>
+        <v>418</v>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Sozialdemokratische Partei der Schweiz</t>
+          <t>IG Nachhaltigkeitsinitiative</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -1203,15 +1203,15 @@
         </is>
       </c>
       <c r="G14" s="6" t="n">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Ablehnung der Abstimmungsvorlage</t>
+          <t>Annahme der Abstimmungsvorlage</t>
         </is>
       </c>
       <c r="I14" s="6" t="n">
-        <v>1563</v>
+        <v>1555</v>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
@@ -1219,10 +1219,10 @@
         </is>
       </c>
       <c r="K14" s="7" t="n">
-        <v>1901724.0</v>
+        <v>6173061.58</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>1890880.0</v>
+        <v>5678238.72</v>
       </c>
       <c r="M14" s="7" t="n">
         <v>0.0</v>
@@ -1231,15 +1231,15 @@
         <v>0.0</v>
       </c>
       <c r="O14" s="7" t="n">
-        <v>10844.0</v>
+        <v>93822.0</v>
       </c>
       <c r="P14" s="7" t="n">
-        <v>0.0</v>
+        <v>401000.86</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3">
-        <v>46248.61550888791</v>
+        <v>46255.35675360831</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
@@ -1250,11 +1250,11 @@
         <v>46187.0</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>59</v>
+        <v>8</v>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Die Mitte</t>
+          <t>Sozialdemokratische Partei der Schweiz</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -1263,7 +1263,7 @@
         </is>
       </c>
       <c r="G15" s="6" t="n">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
@@ -1271,7 +1271,7 @@
         </is>
       </c>
       <c r="I15" s="6" t="n">
-        <v>1566</v>
+        <v>1563</v>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
@@ -1279,10 +1279,10 @@
         </is>
       </c>
       <c r="K15" s="7" t="n">
-        <v>135000.0</v>
+        <v>1901724.0</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>135000.0</v>
+        <v>1890880.0</v>
       </c>
       <c r="M15" s="7" t="n">
         <v>0.0</v>
@@ -1291,7 +1291,7 @@
         <v>0.0</v>
       </c>
       <c r="O15" s="7" t="n">
-        <v>0.0</v>
+        <v>10844.0</v>
       </c>
       <c r="P15" s="7" t="n">
         <v>0.0</v>
@@ -1299,7 +1299,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3">
-        <v>46248.61550888943</v>
+        <v>46255.35675361026</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
@@ -1310,11 +1310,11 @@
         <v>46187.0</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>413</v>
+        <v>59</v>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Handel Schweiz</t>
+          <t>Die Mitte</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
         </is>
       </c>
       <c r="G16" s="6" t="n">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
@@ -1331,7 +1331,7 @@
         </is>
       </c>
       <c r="I16" s="6" t="n">
-        <v>1583</v>
+        <v>1566</v>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
@@ -1339,10 +1339,10 @@
         </is>
       </c>
       <c r="K16" s="7" t="n">
-        <v>91724.0</v>
+        <v>135000.0</v>
       </c>
       <c r="L16" s="7" t="n">
-        <v>0.0</v>
+        <v>135000.0</v>
       </c>
       <c r="M16" s="7" t="n">
         <v>0.0</v>
@@ -1354,12 +1354,12 @@
         <v>0.0</v>
       </c>
       <c r="P16" s="7" t="n">
-        <v>91724.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3">
-        <v>46248.615508891016</v>
+        <v>46255.3567536119</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
@@ -1370,11 +1370,11 @@
         <v>46187.0</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Schweizer Hotelier-Verein (SHV)</t>
+          <t>Schweizerische Flüchtlingshilfe SFH</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -1383,7 +1383,7 @@
         </is>
       </c>
       <c r="G17" s="6" t="n">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
@@ -1391,7 +1391,7 @@
         </is>
       </c>
       <c r="I17" s="6" t="n">
-        <v>1584</v>
+        <v>1587</v>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
@@ -1399,10 +1399,10 @@
         </is>
       </c>
       <c r="K17" s="7" t="n">
-        <v>89311.85</v>
+        <v>303000.0</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>0.0</v>
+        <v>10000.0</v>
       </c>
       <c r="M17" s="7" t="n">
         <v>0.0</v>
@@ -1414,12 +1414,12 @@
         <v>0.0</v>
       </c>
       <c r="P17" s="7" t="n">
-        <v>89311.85</v>
+        <v>293000.0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3">
-        <v>46248.61550889264</v>
+        <v>46255.35675361366</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
@@ -1430,50 +1430,230 @@
         <v>46187.0</v>
       </c>
       <c r="D18" s="6" t="n">
+        <v>457</v>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Junge Schweizerische Volkspartei</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>585</v>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Annahme der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>1585</v>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung der Schlussrechnung über die Einnahmen</t>
+        </is>
+      </c>
+      <c r="K18" s="7" t="n">
+        <v>53395.85</v>
+      </c>
+      <c r="L18" s="7" t="n">
+        <v>37000.0</v>
+      </c>
+      <c r="M18" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N18" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="O18" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="P18" s="7" t="n">
+        <v>16395.85</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3">
+        <v>46255.35675361569</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C19" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>413</v>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Handel Schweiz</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>586</v>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="n">
+        <v>1583</v>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung der Schlussrechnung über die Einnahmen</t>
+        </is>
+      </c>
+      <c r="K19" s="7" t="n">
+        <v>91724.0</v>
+      </c>
+      <c r="L19" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M19" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N19" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="O19" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="P19" s="7" t="n">
+        <v>91724.0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3">
+        <v>46255.35675361763</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C20" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>458</v>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Schweizer Hotelier-Verein (SHV)</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>587</v>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Ablehnung der Abstimmungsvorlage</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>1584</v>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>Offenlegung der Schlussrechnung über die Einnahmen</t>
+        </is>
+      </c>
+      <c r="K20" s="7" t="n">
+        <v>89311.85</v>
+      </c>
+      <c r="L20" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M20" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N20" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="O20" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="P20" s="7" t="n">
+        <v>89311.85</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3">
+        <v>46255.35675361933</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Keine 10-Millionen-Schweiz! (Nachhaltigkeitsinitiative)</t>
+        </is>
+      </c>
+      <c r="C21" s="5">
+        <v>46187.0</v>
+      </c>
+      <c r="D21" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>Sozialdemokratische Partei des Kantons Zürich</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>Juristische Person oder Personengesellschaft</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="n">
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Juristische Person oder Personengesellschaft</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="n">
         <v>588</v>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>Ablehnung der Abstimmungsvorlage</t>
         </is>
       </c>
-      <c r="I18" s="6" t="n">
+      <c r="I21" s="6" t="n">
         <v>1549</v>
       </c>
-      <c r="J18" s="4" t="inlineStr">
+      <c r="J21" s="4" t="inlineStr">
         <is>
           <t>Offenlegung der Schlussrechnung über die Einnahmen</t>
         </is>
       </c>
-      <c r="K18" s="7" t="n">
+      <c r="K21" s="7" t="n">
         <v>68602.3</v>
       </c>
-      <c r="L18" s="7" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="M18" s="7" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="N18" s="7" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="O18" s="7" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="P18" s="7" t="n">
+      <c r="L21" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="M21" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N21" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="O21" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="P21" s="7" t="n">
         <v>68602.3</v>
       </c>
     </row>
@@ -1632,7 +1812,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3">
-        <v>46248.615508895775</v>
+        <v>46255.35675362262</v>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
@@ -1704,7 +1884,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3">
-        <v>46248.615508897645</v>
+        <v>46255.35675362469</v>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
@@ -1776,7 +1956,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3">
-        <v>46248.615508898845</v>
+        <v>46255.35675362604</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
@@ -1848,7 +2028,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3">
-        <v>46248.61550889978</v>
+        <v>46255.356753627435</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
@@ -1920,7 +2100,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3">
-        <v>46248.61550890088</v>
+        <v>46255.35675362857</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
@@ -2000,7 +2180,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3">
-        <v>46248.615508902054</v>
+        <v>46255.35675362992</v>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
@@ -2072,7 +2252,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3">
-        <v>46248.61550890322</v>
+        <v>46255.35675363119</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
@@ -2152,7 +2332,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3">
-        <v>46248.61550890416</v>
+        <v>46255.35675363269</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
@@ -2224,7 +2404,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3">
-        <v>46248.61550890552</v>
+        <v>46255.35675363389</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
@@ -2296,7 +2476,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3">
-        <v>46248.61550890638</v>
+        <v>46255.35675363501</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
@@ -2368,7 +2548,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3">
-        <v>46248.61550890722</v>
+        <v>46255.356753636166</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
@@ -2440,7 +2620,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3">
-        <v>46248.61550890806</v>
+        <v>46255.35675363728</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
@@ -2512,7 +2692,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3">
-        <v>46248.61550890893</v>
+        <v>46255.35675363861</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
@@ -2584,7 +2764,7 @@
     </row>
     <row r="15">
       <c r="A15" s="3">
-        <v>46248.615508909854</v>
+        <v>46255.356753639775</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
@@ -2656,7 +2836,7 @@
     </row>
     <row r="16">
       <c r="A16" s="3">
-        <v>46248.61550891075</v>
+        <v>46255.3567536409</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
@@ -2728,7 +2908,7 @@
     </row>
     <row r="17">
       <c r="A17" s="3">
-        <v>46248.61550891163</v>
+        <v>46255.35675364204</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
@@ -2800,7 +2980,7 @@
     </row>
     <row r="18">
       <c r="A18" s="3">
-        <v>46248.61550891261</v>
+        <v>46255.356753643144</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
@@ -2872,7 +3052,7 @@
     </row>
     <row r="19">
       <c r="A19" s="3">
-        <v>46248.6155089135</v>
+        <v>46255.35675364441</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
@@ -2944,7 +3124,7 @@
     </row>
     <row r="20">
       <c r="A20" s="3">
-        <v>46248.61550891433</v>
+        <v>46255.35675364553</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
@@ -3016,7 +3196,7 @@
     </row>
     <row r="21">
       <c r="A21" s="3">
-        <v>46248.61550891521</v>
+        <v>46255.35675364664</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
@@ -3088,7 +3268,7 @@
     </row>
     <row r="22">
       <c r="A22" s="3">
-        <v>46248.6155089162</v>
+        <v>46255.3567536478</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
@@ -3168,7 +3348,7 @@
     </row>
     <row r="23">
       <c r="A23" s="3">
-        <v>46248.61550891715</v>
+        <v>46255.356753648965</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
@@ -3240,7 +3420,7 @@
     </row>
     <row r="24">
       <c r="A24" s="3">
-        <v>46248.61550891801</v>
+        <v>46255.35675365025</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
@@ -3312,7 +3492,7 @@
     </row>
     <row r="25">
       <c r="A25" s="3">
-        <v>46248.615508918854</v>
+        <v>46255.356753651366</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
@@ -3384,7 +3564,7 @@
     </row>
     <row r="26">
       <c r="A26" s="3">
-        <v>46248.61550891975</v>
+        <v>46255.35675365254</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
@@ -3456,7 +3636,7 @@
     </row>
     <row r="27">
       <c r="A27" s="3">
-        <v>46248.61550892061</v>
+        <v>46255.35675365364</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
@@ -3528,7 +3708,7 @@
     </row>
     <row r="28">
       <c r="A28" s="3">
-        <v>46248.6155089216</v>
+        <v>46255.356753654756</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
@@ -3608,7 +3788,7 @@
     </row>
     <row r="29">
       <c r="A29" s="3">
-        <v>46248.61550892257</v>
+        <v>46255.35675365606</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
@@ -3680,7 +3860,7 @@
     </row>
     <row r="30">
       <c r="A30" s="3">
-        <v>46248.615508923525</v>
+        <v>46255.35675365719</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
@@ -3760,7 +3940,7 @@
     </row>
     <row r="31">
       <c r="A31" s="3">
-        <v>46248.61550892445</v>
+        <v>46255.35675365836</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
@@ -3832,7 +4012,7 @@
     </row>
     <row r="32">
       <c r="A32" s="3">
-        <v>46248.61550892531</v>
+        <v>46255.35675365947</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
@@ -3912,7 +4092,7 @@
     </row>
     <row r="33">
       <c r="A33" s="3">
-        <v>46248.61550892622</v>
+        <v>46255.356753660664</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
@@ -3992,7 +4172,7 @@
     </row>
     <row r="34">
       <c r="A34" s="3">
-        <v>46248.61550892714</v>
+        <v>46255.35675366206</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>

</xml_diff>